<commit_message>
team config table complete
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BEA253B1-4181-430B-B220-E8C8B6FCCC88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930E3BDA-3C74-471C-9850-5DCC8F5D5180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-21697" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="39">
   <si>
     <t>year</t>
   </si>
@@ -131,9 +131,6 @@
     <t>charles leclerc</t>
   </si>
   <si>
-    <t>isaac hadjar</t>
-  </si>
-  <si>
     <t>oliver bearman</t>
   </si>
   <si>
@@ -144,6 +141,21 @@
   </si>
   <si>
     <t>pierre gasly</t>
+  </si>
+  <si>
+    <t>isack hadjar</t>
+  </si>
+  <si>
+    <t>franco colapinto</t>
+  </si>
+  <si>
+    <t>arvid lindblad</t>
+  </si>
+  <si>
+    <t>gabriel bortoleto</t>
+  </si>
+  <si>
+    <t>lance stroll</t>
   </si>
 </sst>
 </file>
@@ -534,6 +546,7 @@
     <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -603,23 +616,53 @@
       <c r="B2">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>16</v>
+      </c>
       <c r="D2" t="s">
         <v>21</v>
       </c>
+      <c r="E2">
+        <v>33</v>
+      </c>
       <c r="F2" t="s">
         <v>24</v>
       </c>
+      <c r="G2">
+        <v>43</v>
+      </c>
       <c r="H2" t="s">
         <v>25</v>
       </c>
+      <c r="I2">
+        <v>10</v>
+      </c>
       <c r="J2" t="s">
         <v>29</v>
       </c>
+      <c r="K2">
+        <v>44</v>
+      </c>
       <c r="L2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2">
+        <v>18</v>
+      </c>
+      <c r="N2" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2">
+        <v>39</v>
+      </c>
+      <c r="P2" t="s">
         <v>32</v>
       </c>
-      <c r="P2" t="s">
-        <v>33</v>
+      <c r="Q2">
+        <v>43</v>
+      </c>
+      <c r="R2" t="s">
+        <v>25</v>
       </c>
       <c r="S2" t="s">
         <v>17</v>
@@ -632,23 +675,53 @@
       <c r="B3">
         <v>1</v>
       </c>
+      <c r="C3">
+        <v>26</v>
+      </c>
       <c r="D3" t="s">
         <v>22</v>
       </c>
+      <c r="E3">
+        <v>33</v>
+      </c>
       <c r="F3" t="s">
         <v>24</v>
       </c>
+      <c r="G3">
+        <v>43</v>
+      </c>
       <c r="H3" t="s">
         <v>25</v>
       </c>
+      <c r="I3">
+        <v>26</v>
+      </c>
       <c r="J3" t="s">
-        <v>30</v>
+        <v>34</v>
+      </c>
+      <c r="K3">
+        <v>44</v>
       </c>
       <c r="L3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3">
+        <v>18</v>
+      </c>
+      <c r="N3" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
         <v>32</v>
       </c>
-      <c r="P3" t="s">
-        <v>33</v>
+      <c r="Q3">
+        <v>43</v>
+      </c>
+      <c r="R3" t="s">
+        <v>25</v>
       </c>
       <c r="S3" t="s">
         <v>18</v>
@@ -661,23 +734,53 @@
       <c r="B4">
         <v>2</v>
       </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
       <c r="D4" t="s">
         <v>23</v>
       </c>
+      <c r="E4">
+        <v>33</v>
+      </c>
       <c r="F4" t="s">
         <v>24</v>
       </c>
+      <c r="G4">
+        <v>43</v>
+      </c>
       <c r="H4" t="s">
         <v>25</v>
       </c>
+      <c r="I4">
+        <v>48</v>
+      </c>
       <c r="J4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4">
+        <v>44</v>
+      </c>
+      <c r="L4" t="s">
         <v>31</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4">
+        <v>18</v>
+      </c>
+      <c r="N4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O4">
+        <v>39</v>
+      </c>
+      <c r="P4" t="s">
         <v>32</v>
       </c>
-      <c r="P4" t="s">
-        <v>33</v>
+      <c r="Q4">
+        <v>43</v>
+      </c>
+      <c r="R4" t="s">
+        <v>25</v>
       </c>
       <c r="S4" t="s">
         <v>17</v>
@@ -690,20 +793,53 @@
       <c r="B5">
         <v>2</v>
       </c>
+      <c r="C5">
+        <v>30</v>
+      </c>
       <c r="D5" t="s">
         <v>23</v>
       </c>
+      <c r="E5">
+        <v>33</v>
+      </c>
       <c r="F5" t="s">
         <v>24</v>
       </c>
+      <c r="G5">
+        <v>43</v>
+      </c>
       <c r="H5" t="s">
         <v>25</v>
       </c>
+      <c r="I5">
+        <v>48</v>
+      </c>
       <c r="J5" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="L5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M5">
+        <v>20</v>
+      </c>
+      <c r="N5" t="s">
+        <v>37</v>
+      </c>
+      <c r="O5">
+        <v>54</v>
       </c>
       <c r="P5" t="s">
-        <v>34</v>
+        <v>33</v>
+      </c>
+      <c r="Q5">
+        <v>43</v>
+      </c>
+      <c r="R5" t="s">
+        <v>25</v>
       </c>
       <c r="S5" t="s">
         <v>18</v>
@@ -716,23 +852,53 @@
       <c r="B6">
         <v>3</v>
       </c>
+      <c r="C6">
+        <v>30</v>
+      </c>
       <c r="D6" t="s">
         <v>23</v>
       </c>
+      <c r="E6">
+        <v>33</v>
+      </c>
       <c r="F6" t="s">
         <v>24</v>
       </c>
+      <c r="G6">
+        <v>22</v>
+      </c>
       <c r="H6" t="s">
         <v>26</v>
       </c>
+      <c r="I6">
+        <v>48</v>
+      </c>
       <c r="J6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6">
+        <v>26</v>
+      </c>
+      <c r="L6" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6">
+        <v>44</v>
+      </c>
+      <c r="N6" t="s">
         <v>31</v>
       </c>
-      <c r="L6" t="s">
-        <v>30</v>
+      <c r="O6">
+        <v>39</v>
       </c>
       <c r="P6" t="s">
-        <v>33</v>
+        <v>32</v>
+      </c>
+      <c r="Q6">
+        <v>22</v>
+      </c>
+      <c r="R6" t="s">
+        <v>26</v>
       </c>
       <c r="S6" t="s">
         <v>17</v>
@@ -745,20 +911,53 @@
       <c r="B7">
         <v>3</v>
       </c>
+      <c r="C7">
+        <v>30</v>
+      </c>
       <c r="D7" t="s">
         <v>23</v>
       </c>
+      <c r="E7">
+        <v>33</v>
+      </c>
       <c r="F7" t="s">
         <v>24</v>
       </c>
+      <c r="G7">
+        <v>51</v>
+      </c>
       <c r="H7" t="s">
         <v>27</v>
       </c>
+      <c r="I7">
+        <v>48</v>
+      </c>
       <c r="J7" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="K7">
+        <v>6</v>
+      </c>
+      <c r="L7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M7">
+        <v>20</v>
+      </c>
+      <c r="N7" t="s">
+        <v>37</v>
+      </c>
+      <c r="O7">
+        <v>54</v>
       </c>
       <c r="P7" t="s">
-        <v>34</v>
+        <v>33</v>
+      </c>
+      <c r="Q7">
+        <v>51</v>
+      </c>
+      <c r="R7" t="s">
+        <v>27</v>
       </c>
       <c r="S7" t="s">
         <v>18</v>
@@ -771,23 +970,53 @@
       <c r="B8">
         <v>6</v>
       </c>
+      <c r="C8">
+        <v>30</v>
+      </c>
       <c r="D8" t="s">
         <v>23</v>
       </c>
+      <c r="E8">
+        <v>33</v>
+      </c>
       <c r="F8" t="s">
         <v>24</v>
       </c>
+      <c r="G8">
+        <v>22</v>
+      </c>
       <c r="H8" t="s">
         <v>26</v>
       </c>
+      <c r="I8">
+        <v>48</v>
+      </c>
       <c r="J8" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="K8">
+        <v>26</v>
       </c>
       <c r="L8" t="s">
-        <v>30</v>
+        <v>34</v>
+      </c>
+      <c r="M8">
+        <v>35</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8">
+        <v>39</v>
       </c>
       <c r="P8" t="s">
-        <v>33</v>
+        <v>32</v>
+      </c>
+      <c r="Q8">
+        <v>22</v>
+      </c>
+      <c r="R8" t="s">
+        <v>26</v>
       </c>
       <c r="S8" t="s">
         <v>17</v>
@@ -800,20 +1029,53 @@
       <c r="B9">
         <v>6</v>
       </c>
+      <c r="C9">
+        <v>30</v>
+      </c>
       <c r="D9" t="s">
         <v>23</v>
       </c>
+      <c r="E9">
+        <v>33</v>
+      </c>
       <c r="F9" t="s">
         <v>24</v>
       </c>
+      <c r="G9">
+        <v>36</v>
+      </c>
       <c r="H9" t="s">
         <v>28</v>
       </c>
+      <c r="I9">
+        <v>48</v>
+      </c>
       <c r="J9" t="s">
+        <v>30</v>
+      </c>
+      <c r="K9">
+        <v>6</v>
+      </c>
+      <c r="L9" t="s">
+        <v>36</v>
+      </c>
+      <c r="M9">
+        <v>54</v>
+      </c>
+      <c r="N9" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9">
+        <v>44</v>
+      </c>
+      <c r="P9" t="s">
         <v>31</v>
       </c>
-      <c r="P9" t="s">
-        <v>32</v>
+      <c r="Q9">
+        <v>36</v>
+      </c>
+      <c r="R9" t="s">
+        <v>28</v>
       </c>
       <c r="S9" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
testing simulation flow for profile 1: max_predicted_points
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930E3BDA-3C74-471C-9850-5DCC8F5D5180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4FBCDD-3652-4417-84CD-50631F7C736C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21697" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="40">
   <si>
     <t>year</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>lance stroll</t>
+  </si>
+  <si>
+    <t>race_id</t>
   </si>
 </sst>
 </file>
@@ -527,557 +530,585 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:S9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5" customWidth="1"/>
+    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.73046875" customWidth="1"/>
+    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.73046875" customWidth="1"/>
+    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>10</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>12</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>14</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>15</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>2026</v>
       </c>
       <c r="B2">
+        <v>73</v>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>21</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>33</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>24</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>43</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>25</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>10</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>29</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>44</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>31</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>18</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>35</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>39</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>43</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>25</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2026</v>
       </c>
       <c r="B3">
+        <v>73</v>
+      </c>
+      <c r="C3">
         <v>1</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>26</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>33</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>24</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>43</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>25</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>26</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>34</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>44</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>31</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>18</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>35</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>39</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>32</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>43</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>25</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2026</v>
       </c>
       <c r="B4">
+        <v>74</v>
+      </c>
+      <c r="C4">
         <v>2</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>30</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>23</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>33</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>43</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>25</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>48</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>30</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>44</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>31</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>18</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>35</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>39</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>32</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>43</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>25</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2026</v>
       </c>
       <c r="B5">
+        <v>74</v>
+      </c>
+      <c r="C5">
         <v>2</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>23</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>33</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>24</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>43</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>25</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>48</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>30</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>6</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>36</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>20</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>37</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>54</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>33</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>43</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>25</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2026</v>
       </c>
       <c r="B6">
+        <v>75</v>
+      </c>
+      <c r="C6">
         <v>3</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>30</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>23</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>33</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>24</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>22</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>26</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>48</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>30</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>26</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>34</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>44</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>31</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>39</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>32</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>22</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>26</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2026</v>
       </c>
       <c r="B7">
+        <v>75</v>
+      </c>
+      <c r="C7">
         <v>3</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>30</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>23</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>33</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>24</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>51</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>27</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>48</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>30</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>6</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>36</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>20</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>37</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>54</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>33</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>51</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>27</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2026</v>
       </c>
       <c r="B8">
+        <v>76</v>
+      </c>
+      <c r="C8">
         <v>6</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>30</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>23</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>33</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>24</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>22</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>26</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>48</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>30</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>26</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>34</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>35</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>38</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>39</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>32</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>22</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>26</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2026</v>
       </c>
       <c r="B9">
+        <v>76</v>
+      </c>
+      <c r="C9">
         <v>6</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>30</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>23</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>33</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>24</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>36</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>28</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>48</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>30</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>6</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>36</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>54</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>33</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>44</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>31</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>36</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>28</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
moving older files and folders to deprecated folders
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4FBCDD-3652-4417-84CD-50631F7C736C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18457973-99BA-422D-9018-EFFAAE471538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="43">
   <si>
     <t>year</t>
   </si>
@@ -159,6 +159,15 @@
   </si>
   <si>
     <t>race_id</t>
+  </si>
+  <si>
+    <t>valtteri bottas</t>
+  </si>
+  <si>
+    <t>sergio perez</t>
+  </si>
+  <si>
+    <t>kimi antonelli</t>
   </si>
 </sst>
 </file>
@@ -530,31 +539,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:T11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.73046875" customWidth="1"/>
-    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.73046875" customWidth="1"/>
-    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -616,7 +625,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -678,7 +687,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -740,7 +749,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -802,7 +811,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -864,7 +873,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -926,7 +935,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -988,7 +997,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -1050,7 +1059,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -1109,6 +1118,130 @@
         <v>28</v>
       </c>
       <c r="T9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2026</v>
+      </c>
+      <c r="B10">
+        <v>77</v>
+      </c>
+      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10">
+        <v>30</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10">
+        <v>16</v>
+      </c>
+      <c r="G10" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10">
+        <v>22</v>
+      </c>
+      <c r="I10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10">
+        <v>20</v>
+      </c>
+      <c r="K10" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10">
+        <v>44</v>
+      </c>
+      <c r="M10" t="s">
+        <v>31</v>
+      </c>
+      <c r="N10">
+        <v>35</v>
+      </c>
+      <c r="O10" t="s">
+        <v>38</v>
+      </c>
+      <c r="P10">
+        <v>66</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>40</v>
+      </c>
+      <c r="R10">
+        <v>22</v>
+      </c>
+      <c r="S10" t="s">
+        <v>26</v>
+      </c>
+      <c r="T10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2026</v>
+      </c>
+      <c r="B11">
+        <v>77</v>
+      </c>
+      <c r="C11">
+        <v>7</v>
+      </c>
+      <c r="D11">
+        <v>30</v>
+      </c>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11">
+        <v>33</v>
+      </c>
+      <c r="G11" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11">
+        <v>34</v>
+      </c>
+      <c r="I11" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11">
+        <v>39</v>
+      </c>
+      <c r="K11" t="s">
+        <v>32</v>
+      </c>
+      <c r="L11">
+        <v>54</v>
+      </c>
+      <c r="M11" t="s">
+        <v>33</v>
+      </c>
+      <c r="N11">
+        <v>60</v>
+      </c>
+      <c r="O11" t="s">
+        <v>41</v>
+      </c>
+      <c r="P11">
+        <v>48</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>30</v>
+      </c>
+      <c r="R11">
+        <v>34</v>
+      </c>
+      <c r="S11" t="s">
+        <v>42</v>
+      </c>
+      <c r="T11" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
pre barcelona db update
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18457973-99BA-422D-9018-EFFAAE471538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A91C5BA-CFF0-4CDB-A724-029F22655407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="45">
   <si>
     <t>year</t>
   </si>
@@ -168,6 +168,12 @@
   </si>
   <si>
     <t>kimi antonelli</t>
+  </si>
+  <si>
+    <t>Audi</t>
+  </si>
+  <si>
+    <t>lewis hamilton</t>
   </si>
 </sst>
 </file>
@@ -539,31 +545,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T13"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.73046875" customWidth="1"/>
+    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.73046875" customWidth="1"/>
+    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -625,7 +631,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -687,7 +693,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -749,7 +755,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -811,7 +817,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -873,7 +879,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -935,7 +941,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -997,7 +1003,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -1059,7 +1065,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -1121,7 +1127,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -1183,7 +1189,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -1242,6 +1248,127 @@
         <v>42</v>
       </c>
       <c r="T11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>2026</v>
+      </c>
+      <c r="B12">
+        <v>78</v>
+      </c>
+      <c r="C12">
+        <v>8</v>
+      </c>
+      <c r="D12">
+        <v>30</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>43</v>
+      </c>
+      <c r="H12">
+        <v>22</v>
+      </c>
+      <c r="I12" t="s">
+        <v>26</v>
+      </c>
+      <c r="J12">
+        <v>34</v>
+      </c>
+      <c r="K12" t="s">
+        <v>42</v>
+      </c>
+      <c r="L12">
+        <v>44</v>
+      </c>
+      <c r="M12" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12">
+        <v>35</v>
+      </c>
+      <c r="O12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P12">
+        <v>20</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>37</v>
+      </c>
+      <c r="R12">
+        <v>22</v>
+      </c>
+      <c r="S12" t="s">
+        <v>26</v>
+      </c>
+      <c r="T12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>2026</v>
+      </c>
+      <c r="B13">
+        <v>78</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13">
+        <v>11</v>
+      </c>
+      <c r="G13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H13">
+        <v>34</v>
+      </c>
+      <c r="I13" t="s">
+        <v>42</v>
+      </c>
+      <c r="K13" t="s">
+        <v>44</v>
+      </c>
+      <c r="L13">
+        <v>66</v>
+      </c>
+      <c r="M13" t="s">
+        <v>40</v>
+      </c>
+      <c r="N13">
+        <v>35</v>
+      </c>
+      <c r="O13" t="s">
+        <v>38</v>
+      </c>
+      <c r="P13">
+        <v>39</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>32</v>
+      </c>
+      <c r="R13">
+        <v>34</v>
+      </c>
+      <c r="S13" t="s">
+        <v>42</v>
+      </c>
+      <c r="T13" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
post barcelona results added
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A91C5BA-CFF0-4CDB-A724-029F22655407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACB6099A-4A94-42F9-8CE8-0C595F7D0C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="45">
   <si>
     <t>year</t>
   </si>
@@ -545,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T13"/>
+  <dimension ref="A1:T15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -1341,6 +1341,9 @@
       <c r="I13" t="s">
         <v>42</v>
       </c>
+      <c r="J13">
+        <v>38</v>
+      </c>
       <c r="K13" t="s">
         <v>44</v>
       </c>
@@ -1369,6 +1372,130 @@
         <v>42</v>
       </c>
       <c r="T13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>2026</v>
+      </c>
+      <c r="B14">
+        <v>79</v>
+      </c>
+      <c r="C14">
+        <v>9</v>
+      </c>
+      <c r="D14">
+        <v>30</v>
+      </c>
+      <c r="E14" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14">
+        <v>11</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
+      <c r="H14">
+        <v>34</v>
+      </c>
+      <c r="I14" t="s">
+        <v>42</v>
+      </c>
+      <c r="J14">
+        <v>26</v>
+      </c>
+      <c r="K14" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14">
+        <v>44</v>
+      </c>
+      <c r="M14" t="s">
+        <v>31</v>
+      </c>
+      <c r="N14">
+        <v>38</v>
+      </c>
+      <c r="O14" t="s">
+        <v>44</v>
+      </c>
+      <c r="P14">
+        <v>20</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>37</v>
+      </c>
+      <c r="R14">
+        <v>34</v>
+      </c>
+      <c r="S14" t="s">
+        <v>42</v>
+      </c>
+      <c r="T14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A15">
+        <v>2026</v>
+      </c>
+      <c r="B15">
+        <v>79</v>
+      </c>
+      <c r="C15">
+        <v>9</v>
+      </c>
+      <c r="D15">
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15">
+        <v>11</v>
+      </c>
+      <c r="G15" t="s">
+        <v>43</v>
+      </c>
+      <c r="H15">
+        <v>34</v>
+      </c>
+      <c r="I15" t="s">
+        <v>42</v>
+      </c>
+      <c r="J15">
+        <v>22</v>
+      </c>
+      <c r="K15" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15">
+        <v>44</v>
+      </c>
+      <c r="M15" t="s">
+        <v>31</v>
+      </c>
+      <c r="N15">
+        <v>20</v>
+      </c>
+      <c r="O15" t="s">
+        <v>37</v>
+      </c>
+      <c r="P15">
+        <v>66</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>40</v>
+      </c>
+      <c r="R15">
+        <v>34</v>
+      </c>
+      <c r="S15" t="s">
+        <v>42</v>
+      </c>
+      <c r="T15" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updating manual data from austria
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACB6099A-4A94-42F9-8CE8-0C595F7D0C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{247F19CB-F01D-4A98-8206-5DCCC1AB91E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="45">
   <si>
     <t>year</t>
   </si>
@@ -545,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -1499,6 +1499,130 @@
         <v>18</v>
       </c>
     </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>2026</v>
+      </c>
+      <c r="B16">
+        <v>80</v>
+      </c>
+      <c r="C16">
+        <v>10</v>
+      </c>
+      <c r="D16">
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16">
+        <v>34</v>
+      </c>
+      <c r="I16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J16">
+        <v>26</v>
+      </c>
+      <c r="K16" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16">
+        <v>44</v>
+      </c>
+      <c r="M16" t="s">
+        <v>31</v>
+      </c>
+      <c r="N16">
+        <v>38</v>
+      </c>
+      <c r="O16" t="s">
+        <v>44</v>
+      </c>
+      <c r="P16">
+        <v>20</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>37</v>
+      </c>
+      <c r="R16">
+        <v>34</v>
+      </c>
+      <c r="S16" t="s">
+        <v>42</v>
+      </c>
+      <c r="T16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A17">
+        <v>2026</v>
+      </c>
+      <c r="B17">
+        <v>80</v>
+      </c>
+      <c r="C17">
+        <v>10</v>
+      </c>
+      <c r="D17">
+        <v>30</v>
+      </c>
+      <c r="E17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17">
+        <v>11</v>
+      </c>
+      <c r="G17" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17">
+        <v>34</v>
+      </c>
+      <c r="I17" t="s">
+        <v>42</v>
+      </c>
+      <c r="J17">
+        <v>22</v>
+      </c>
+      <c r="K17" t="s">
+        <v>26</v>
+      </c>
+      <c r="L17">
+        <v>44</v>
+      </c>
+      <c r="M17" t="s">
+        <v>31</v>
+      </c>
+      <c r="N17">
+        <v>20</v>
+      </c>
+      <c r="O17" t="s">
+        <v>37</v>
+      </c>
+      <c r="P17">
+        <v>66</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>40</v>
+      </c>
+      <c r="R17">
+        <v>34</v>
+      </c>
+      <c r="S17" t="s">
+        <v>42</v>
+      </c>
+      <c r="T17" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
new data for belgium
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{247F19CB-F01D-4A98-8206-5DCCC1AB91E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C2AE25-DFB9-4D53-BB1B-BE466216EE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="45">
   <si>
     <t>year</t>
   </si>
@@ -545,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -1623,6 +1623,130 @@
         <v>18</v>
       </c>
     </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A18">
+        <v>2026</v>
+      </c>
+      <c r="B18">
+        <v>81</v>
+      </c>
+      <c r="C18">
+        <v>11</v>
+      </c>
+      <c r="D18">
+        <v>30</v>
+      </c>
+      <c r="E18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18">
+        <v>11</v>
+      </c>
+      <c r="G18" t="s">
+        <v>43</v>
+      </c>
+      <c r="H18">
+        <v>34</v>
+      </c>
+      <c r="I18" t="s">
+        <v>42</v>
+      </c>
+      <c r="J18">
+        <v>26</v>
+      </c>
+      <c r="K18" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18">
+        <v>44</v>
+      </c>
+      <c r="M18" t="s">
+        <v>31</v>
+      </c>
+      <c r="N18">
+        <v>38</v>
+      </c>
+      <c r="O18" t="s">
+        <v>44</v>
+      </c>
+      <c r="P18">
+        <v>20</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>37</v>
+      </c>
+      <c r="R18">
+        <v>34</v>
+      </c>
+      <c r="S18" t="s">
+        <v>42</v>
+      </c>
+      <c r="T18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A19">
+        <v>2026</v>
+      </c>
+      <c r="B19">
+        <v>81</v>
+      </c>
+      <c r="C19">
+        <v>11</v>
+      </c>
+      <c r="D19">
+        <v>30</v>
+      </c>
+      <c r="E19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19">
+        <v>34</v>
+      </c>
+      <c r="I19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J19">
+        <v>22</v>
+      </c>
+      <c r="K19" t="s">
+        <v>26</v>
+      </c>
+      <c r="L19">
+        <v>44</v>
+      </c>
+      <c r="M19" t="s">
+        <v>31</v>
+      </c>
+      <c r="N19">
+        <v>20</v>
+      </c>
+      <c r="O19" t="s">
+        <v>37</v>
+      </c>
+      <c r="P19">
+        <v>66</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>40</v>
+      </c>
+      <c r="R19">
+        <v>34</v>
+      </c>
+      <c r="S19" t="s">
+        <v>42</v>
+      </c>
+      <c r="T19" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
full pipleline run for hungary
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C2AE25-DFB9-4D53-BB1B-BE466216EE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F353177-89E4-4D39-A350-BD8F0A3C2B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="46">
   <si>
     <t>year</t>
   </si>
@@ -174,6 +174,9 @@
   </si>
   <si>
     <t>lewis hamilton</t>
+  </si>
+  <si>
+    <t>alexander albon</t>
   </si>
 </sst>
 </file>
@@ -545,31 +548,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T19"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:T21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.73046875" customWidth="1"/>
-    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.73046875" customWidth="1"/>
-    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -631,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -693,7 +696,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -755,7 +758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -817,7 +820,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -879,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -941,7 +944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -1003,7 +1006,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -1065,7 +1068,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -1127,7 +1130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -1189,7 +1192,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -1251,7 +1254,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -1313,7 +1316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -1375,7 +1378,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -1437,7 +1440,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -1499,7 +1502,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -1561,7 +1564,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -1623,7 +1626,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -1685,7 +1688,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -1744,6 +1747,130 @@
         <v>42</v>
       </c>
       <c r="T19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2026</v>
+      </c>
+      <c r="B20">
+        <v>82</v>
+      </c>
+      <c r="C20">
+        <v>12</v>
+      </c>
+      <c r="D20">
+        <v>30</v>
+      </c>
+      <c r="E20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20">
+        <v>11</v>
+      </c>
+      <c r="G20" t="s">
+        <v>43</v>
+      </c>
+      <c r="H20">
+        <v>34</v>
+      </c>
+      <c r="I20" t="s">
+        <v>42</v>
+      </c>
+      <c r="J20">
+        <v>26</v>
+      </c>
+      <c r="K20" t="s">
+        <v>34</v>
+      </c>
+      <c r="L20">
+        <v>44</v>
+      </c>
+      <c r="M20" t="s">
+        <v>31</v>
+      </c>
+      <c r="N20">
+        <v>38</v>
+      </c>
+      <c r="O20" t="s">
+        <v>44</v>
+      </c>
+      <c r="P20">
+        <v>6</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>36</v>
+      </c>
+      <c r="R20">
+        <v>34</v>
+      </c>
+      <c r="S20" t="s">
+        <v>42</v>
+      </c>
+      <c r="T20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2026</v>
+      </c>
+      <c r="B21">
+        <v>82</v>
+      </c>
+      <c r="C21">
+        <v>12</v>
+      </c>
+      <c r="D21">
+        <v>30</v>
+      </c>
+      <c r="E21" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21">
+        <v>11</v>
+      </c>
+      <c r="G21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H21">
+        <v>34</v>
+      </c>
+      <c r="I21" t="s">
+        <v>42</v>
+      </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
+      <c r="K21" t="s">
+        <v>45</v>
+      </c>
+      <c r="L21">
+        <v>10</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21">
+        <v>6</v>
+      </c>
+      <c r="O21" t="s">
+        <v>36</v>
+      </c>
+      <c r="P21">
+        <v>44</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>31</v>
+      </c>
+      <c r="R21">
+        <v>34</v>
+      </c>
+      <c r="S21" t="s">
+        <v>42</v>
+      </c>
+      <c r="T21" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated manual data / checked training tables
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F353177-89E4-4D39-A350-BD8F0A3C2B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCBFEF3A-978C-4642-A1AA-44902345A70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-10882" yWindow="-52" windowWidth="10965" windowHeight="12862" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="46">
   <si>
     <t>year</t>
   </si>
@@ -548,31 +548,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.73046875" customWidth="1"/>
+    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.73046875" customWidth="1"/>
+    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -634,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -758,7 +758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -820,7 +820,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -882,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>2026</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>2026</v>
       </c>
@@ -1871,6 +1871,254 @@
         <v>42</v>
       </c>
       <c r="T21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A22">
+        <v>2026</v>
+      </c>
+      <c r="B22">
+        <v>83</v>
+      </c>
+      <c r="C22">
+        <v>12</v>
+      </c>
+      <c r="D22">
+        <v>30</v>
+      </c>
+      <c r="E22" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22">
+        <v>11</v>
+      </c>
+      <c r="G22" t="s">
+        <v>43</v>
+      </c>
+      <c r="H22">
+        <v>34</v>
+      </c>
+      <c r="I22" t="s">
+        <v>42</v>
+      </c>
+      <c r="J22">
+        <v>26</v>
+      </c>
+      <c r="K22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L22">
+        <v>44</v>
+      </c>
+      <c r="M22" t="s">
+        <v>31</v>
+      </c>
+      <c r="N22">
+        <v>38</v>
+      </c>
+      <c r="O22" t="s">
+        <v>44</v>
+      </c>
+      <c r="P22">
+        <v>6</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>36</v>
+      </c>
+      <c r="R22">
+        <v>34</v>
+      </c>
+      <c r="S22" t="s">
+        <v>42</v>
+      </c>
+      <c r="T22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A23">
+        <v>2026</v>
+      </c>
+      <c r="B23">
+        <v>83</v>
+      </c>
+      <c r="C23">
+        <v>12</v>
+      </c>
+      <c r="D23">
+        <v>30</v>
+      </c>
+      <c r="E23" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23">
+        <v>11</v>
+      </c>
+      <c r="G23" t="s">
+        <v>43</v>
+      </c>
+      <c r="H23">
+        <v>34</v>
+      </c>
+      <c r="I23" t="s">
+        <v>42</v>
+      </c>
+      <c r="J23">
+        <v>2</v>
+      </c>
+      <c r="K23" t="s">
+        <v>45</v>
+      </c>
+      <c r="L23">
+        <v>10</v>
+      </c>
+      <c r="M23" t="s">
+        <v>29</v>
+      </c>
+      <c r="N23">
+        <v>6</v>
+      </c>
+      <c r="O23" t="s">
+        <v>36</v>
+      </c>
+      <c r="P23">
+        <v>44</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>31</v>
+      </c>
+      <c r="R23">
+        <v>34</v>
+      </c>
+      <c r="S23" t="s">
+        <v>42</v>
+      </c>
+      <c r="T23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A24">
+        <v>2026</v>
+      </c>
+      <c r="B24">
+        <v>84</v>
+      </c>
+      <c r="C24">
+        <v>13</v>
+      </c>
+      <c r="D24">
+        <v>30</v>
+      </c>
+      <c r="E24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24">
+        <v>11</v>
+      </c>
+      <c r="G24" t="s">
+        <v>43</v>
+      </c>
+      <c r="H24">
+        <v>34</v>
+      </c>
+      <c r="I24" t="s">
+        <v>42</v>
+      </c>
+      <c r="J24">
+        <v>26</v>
+      </c>
+      <c r="K24" t="s">
+        <v>34</v>
+      </c>
+      <c r="L24">
+        <v>44</v>
+      </c>
+      <c r="M24" t="s">
+        <v>31</v>
+      </c>
+      <c r="N24">
+        <v>38</v>
+      </c>
+      <c r="O24" t="s">
+        <v>44</v>
+      </c>
+      <c r="P24">
+        <v>6</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>36</v>
+      </c>
+      <c r="R24">
+        <v>34</v>
+      </c>
+      <c r="S24" t="s">
+        <v>42</v>
+      </c>
+      <c r="T24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A25">
+        <v>2026</v>
+      </c>
+      <c r="B25">
+        <v>84</v>
+      </c>
+      <c r="C25">
+        <v>13</v>
+      </c>
+      <c r="D25">
+        <v>30</v>
+      </c>
+      <c r="E25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25">
+        <v>11</v>
+      </c>
+      <c r="G25" t="s">
+        <v>43</v>
+      </c>
+      <c r="H25">
+        <v>34</v>
+      </c>
+      <c r="I25" t="s">
+        <v>42</v>
+      </c>
+      <c r="J25">
+        <v>2</v>
+      </c>
+      <c r="K25" t="s">
+        <v>45</v>
+      </c>
+      <c r="L25">
+        <v>10</v>
+      </c>
+      <c r="M25" t="s">
+        <v>29</v>
+      </c>
+      <c r="N25">
+        <v>6</v>
+      </c>
+      <c r="O25" t="s">
+        <v>36</v>
+      </c>
+      <c r="P25">
+        <v>44</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>31</v>
+      </c>
+      <c r="R25">
+        <v>34</v>
+      </c>
+      <c r="S25" t="s">
+        <v>42</v>
+      </c>
+      <c r="T25" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
post Dutch GP DB updates
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCBFEF3A-978C-4642-A1AA-44902345A70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D33ABD5-442B-4BCE-A42B-25909ACEA6FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10882" yWindow="-52" windowWidth="10965" windowHeight="12862" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -549,30 +549,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
   <dimension ref="A1:T25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.73046875" customWidth="1"/>
-    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.73046875" customWidth="1"/>
-    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -634,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -758,7 +758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -820,7 +820,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -882,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2026</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2026</v>
       </c>
@@ -1874,7 +1874,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2026</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>83</v>
       </c>
       <c r="C22">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D22">
         <v>30</v>
@@ -1936,7 +1936,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2026</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>83</v>
       </c>
       <c r="C23">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D23">
         <v>30</v>
@@ -1998,7 +1998,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2026</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>84</v>
       </c>
       <c r="C24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D24">
         <v>30</v>
@@ -2027,10 +2027,10 @@
         <v>42</v>
       </c>
       <c r="J24">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="K24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L24">
         <v>44</v>
@@ -2060,7 +2060,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2026</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>84</v>
       </c>
       <c r="C25">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D25">
         <v>30</v>

</xml_diff>

<commit_message>
added italy fantasy data
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36835B59-CF74-4F13-B160-BAB704D1BCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64F5F30-B3E1-472C-8266-457FA009831F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="3045" yWindow="3472" windowWidth="16200" windowHeight="9308" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="46">
   <si>
     <t>year</t>
   </si>
@@ -548,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:T27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -2122,6 +2122,130 @@
         <v>18</v>
       </c>
     </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A26">
+        <v>2026</v>
+      </c>
+      <c r="B26">
+        <v>85</v>
+      </c>
+      <c r="C26">
+        <v>15</v>
+      </c>
+      <c r="D26">
+        <v>30</v>
+      </c>
+      <c r="E26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26">
+        <v>11</v>
+      </c>
+      <c r="G26" t="s">
+        <v>43</v>
+      </c>
+      <c r="H26">
+        <v>35</v>
+      </c>
+      <c r="I26" t="s">
+        <v>42</v>
+      </c>
+      <c r="J26">
+        <v>55</v>
+      </c>
+      <c r="K26" t="s">
+        <v>33</v>
+      </c>
+      <c r="L26">
+        <v>45</v>
+      </c>
+      <c r="M26" t="s">
+        <v>31</v>
+      </c>
+      <c r="N26">
+        <v>39</v>
+      </c>
+      <c r="O26" t="s">
+        <v>44</v>
+      </c>
+      <c r="P26">
+        <v>6</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>36</v>
+      </c>
+      <c r="R26">
+        <v>35</v>
+      </c>
+      <c r="S26" t="s">
+        <v>42</v>
+      </c>
+      <c r="T26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A27">
+        <v>2026</v>
+      </c>
+      <c r="B27">
+        <v>85</v>
+      </c>
+      <c r="C27">
+        <v>15</v>
+      </c>
+      <c r="D27">
+        <v>30</v>
+      </c>
+      <c r="E27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27">
+        <v>11</v>
+      </c>
+      <c r="G27" t="s">
+        <v>43</v>
+      </c>
+      <c r="H27">
+        <v>35</v>
+      </c>
+      <c r="I27" t="s">
+        <v>42</v>
+      </c>
+      <c r="J27">
+        <v>2</v>
+      </c>
+      <c r="K27" t="s">
+        <v>45</v>
+      </c>
+      <c r="L27">
+        <v>10</v>
+      </c>
+      <c r="M27" t="s">
+        <v>29</v>
+      </c>
+      <c r="N27">
+        <v>6</v>
+      </c>
+      <c r="O27" t="s">
+        <v>36</v>
+      </c>
+      <c r="P27">
+        <v>45</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>31</v>
+      </c>
+      <c r="R27">
+        <v>35</v>
+      </c>
+      <c r="S27" t="s">
+        <v>42</v>
+      </c>
+      <c r="T27" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>